<commit_message>
fix(recon): template headers must match parser (\"Invoice No\" not \"invoice_no\")
The XLSX parser expects the human-readable column headers
(\"Invoice No\", \"Supplier BIN\", \"Taxable Amount (BDT)\", …) — see
backend/app/reconciliation/parser.py _PURCHASE_COLUMNS / _SUPPLIER_COLUMNS.

The starter templates and the FileDropzone help-text used snake_case
which would have caused INVALID_XLSX_FORMAT 400s for any user who used
them as-is. Smoke-tested the full POST → parse → match → persist
pipeline with the corrected headers; pipeline returns 201 with proper
aggregates.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/templates/purchase-register-template.xlsx
+++ b/frontend/public/templates/purchase-register-template.xlsx
@@ -427,32 +427,32 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>invoice_no</t>
+          <t>Invoice No</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>supplier_bin</t>
+          <t>Supplier BIN</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>supplier_name</t>
+          <t>Supplier Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>invoice_date</t>
+          <t>Invoice Date</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>taxable_amount_bdt</t>
+          <t>Taxable Amount (BDT)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>vat_amount_bdt</t>
+          <t>VAT Amount (BDT)</t>
         </is>
       </c>
     </row>

</xml_diff>